<commit_message>
updated schedule with optional review session
</commit_message>
<xml_diff>
--- a/course/assets/student-schedule.xlsx
+++ b/course/assets/student-schedule.xlsx
@@ -16,7 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="26">
+  <numFmts count="27">
     <numFmt numFmtId="164" formatCode="&quot;D01 - &quot;ddd\ d\ mmm\ yyyy"/>
     <numFmt numFmtId="165" formatCode="&quot;D02 - &quot;ddd\ d\ mmm\ yyyy"/>
     <numFmt numFmtId="166" formatCode="&quot;D03 - &quot;ddd\ d\ mmm\ yyyy"/>
@@ -43,6 +43,7 @@
     <numFmt numFmtId="187" formatCode="&quot;D24 - &quot;ddd\ d\ mmm\ yyyy"/>
     <numFmt numFmtId="188" formatCode="&quot;D25 - &quot;ddd\ d\ mmm\ yyyy"/>
     <numFmt numFmtId="189" formatCode="&quot;D26 - &quot;ddd\ d\ mmm\ yyyy"/>
+    <numFmt numFmtId="190" formatCode="&quot;Optional - &quot;ddd\ d\ mmm\ yyyy"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -87,7 +88,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -116,6 +117,16 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFEEF1F5"/>
         <bgColor rgb="FFE7F4EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF4C2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4F7FB"/>
       </patternFill>
     </fill>
   </fills>
@@ -175,7 +186,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -380,6 +391,66 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="190" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="173" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="175" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="185" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="187" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="189" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="190" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="20">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -594,7 +665,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StudentScheduleTable" displayName="StudentScheduleTable" ref="A1:F27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StudentScheduleTable" displayName="StudentScheduleTable" ref="A1:F28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A1:F27"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Date"/>
@@ -783,7 +854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="23" customWidth="1" style="34" min="1" max="1"/>
@@ -839,7 +910,7 @@
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/01-data-foundations/README.md","Data foundations")</f>
         <v/>
       </c>
-      <c r="D2" s="41" t="inlineStr">
+      <c r="D2" s="69" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -856,29 +927,29 @@
       </c>
     </row>
     <row r="3" ht="34" customHeight="1" s="35">
-      <c r="A3" s="42" t="n">
+      <c r="A3" s="70" t="n">
         <v>46286</v>
       </c>
-      <c r="B3" s="43" t="inlineStr">
+      <c r="B3" s="71" t="inlineStr">
         <is>
           <t>Where data lives and cloud fundamentals</t>
         </is>
       </c>
-      <c r="C3" s="43">
+      <c r="C3" s="71">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/01-data-foundations/README.md","Data foundations")</f>
         <v/>
       </c>
-      <c r="D3" s="41" t="inlineStr">
+      <c r="D3" s="72" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E3" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F3" s="43" t="inlineStr">
+      <c r="E3" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F3" s="71" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -897,7 +968,7 @@
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/02-sql/README.md","SQL")</f>
         <v/>
       </c>
-      <c r="D4" s="41" t="inlineStr">
+      <c r="D4" s="69" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -914,29 +985,29 @@
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" s="35">
-      <c r="A5" s="45" t="n">
+      <c r="A5" s="73" t="n">
         <v>46293</v>
       </c>
-      <c r="B5" s="43" t="inlineStr">
+      <c r="B5" s="71" t="inlineStr">
         <is>
           <t>SQL foundations continued; aggregation begins</t>
         </is>
       </c>
-      <c r="C5" s="43">
+      <c r="C5" s="71">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/02-sql/README.md","SQL")</f>
         <v/>
       </c>
-      <c r="D5" s="41" t="inlineStr">
+      <c r="D5" s="72" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E5" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F5" s="43" t="inlineStr">
+      <c r="E5" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="71" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -955,7 +1026,7 @@
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/02-sql/README.md","SQL")</f>
         <v/>
       </c>
-      <c r="D6" s="41" t="inlineStr">
+      <c r="D6" s="69" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -972,29 +1043,29 @@
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" s="35">
-      <c r="A7" s="47" t="n">
+      <c r="A7" s="74" t="n">
         <v>46299</v>
       </c>
-      <c r="B7" s="43" t="inlineStr">
+      <c r="B7" s="71" t="inlineStr">
         <is>
           <t>Joins: combining tables</t>
         </is>
       </c>
-      <c r="C7" s="43">
+      <c r="C7" s="71">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/02-sql/README.md","SQL")</f>
         <v/>
       </c>
-      <c r="D7" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E7" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="43" t="inlineStr">
+      <c r="D7" s="72" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E7" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="71" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1013,7 +1084,7 @@
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/02-sql/README.md","SQL")</f>
         <v/>
       </c>
-      <c r="D8" s="41" t="inlineStr">
+      <c r="D8" s="69" t="inlineStr">
         <is>
           <t>After class</t>
         </is>
@@ -1030,551 +1101,580 @@
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" s="35">
-      <c r="A9" s="49" t="n">
+      <c r="A9" s="75" t="n">
         <v>46302</v>
       </c>
-      <c r="B9" s="43" t="inlineStr">
+      <c r="B9" s="71" t="inlineStr">
         <is>
           <t>Subqueries, CTEs and views</t>
         </is>
       </c>
-      <c r="C9" s="43">
+      <c r="C9" s="71">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/02-sql/README.md","SQL")</f>
         <v/>
       </c>
-      <c r="D9" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E9" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F9" s="43" t="inlineStr">
+      <c r="D9" s="72" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E9" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="71" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" s="35">
-      <c r="A10" s="50" t="n">
+      <c r="A10" s="88" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B10" s="77" t="inlineStr">
+        <is>
+          <t>Optional review: SQL so far (D03–D08), 4:00–6:00 PM</t>
+        </is>
+      </c>
+      <c r="C10" s="77">
+        <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/02-sql/README.md","SQL")</f>
+        <v/>
+      </c>
+      <c r="D10" s="78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E10" s="77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F10" s="77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1" s="35">
+      <c r="A11" s="50" t="n">
         <v>46306</v>
       </c>
-      <c r="B10" s="40" t="inlineStr">
+      <c r="B11" s="40" t="inlineStr">
         <is>
           <t>Window functions and SQL wrap-up</t>
         </is>
       </c>
-      <c r="C10" s="40">
+      <c r="C11" s="40">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/02-sql/README.md","SQL")</f>
         <v/>
       </c>
-      <c r="D10" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E10" s="40" t="inlineStr">
+      <c r="D11" s="69" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E11" s="40" t="inlineStr">
         <is>
           <t>Assignment 1</t>
         </is>
       </c>
-      <c r="F10" s="40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1" s="35">
-      <c r="A11" s="51" t="n">
+      <c r="F11" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1" s="35">
+      <c r="A12" s="79" t="n">
         <v>46307</v>
       </c>
-      <c r="B11" s="43" t="inlineStr">
+      <c r="B12" s="71" t="inlineStr">
         <is>
           <t>Machine learning 1: what learning means, and regression</t>
         </is>
       </c>
-      <c r="C11" s="43">
+      <c r="C12" s="71">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/07-machine-learning-and-ai/README.md","Machine learning and AI literacy")</f>
         <v/>
       </c>
-      <c r="D11" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E11" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1" s="35">
-      <c r="A12" s="52" t="n">
+      <c r="D12" s="72" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E12" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1" s="35">
+      <c r="A13" s="52" t="n">
         <v>46313</v>
       </c>
-      <c r="B12" s="40" t="inlineStr">
+      <c r="B13" s="40" t="inlineStr">
         <is>
           <t>Machine learning 2: classification and choosing an algorithm</t>
         </is>
       </c>
-      <c r="C12" s="40">
+      <c r="C13" s="40">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/07-machine-learning-and-ai/README.md","Machine learning and AI literacy")</f>
         <v/>
       </c>
-      <c r="D12" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E12" s="40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F12" s="40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1" s="35">
-      <c r="A13" s="53" t="n">
+      <c r="D13" s="69" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E13" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1" s="35">
+      <c r="A14" s="80" t="n">
         <v>46314</v>
       </c>
-      <c r="B13" s="43" t="inlineStr">
+      <c r="B14" s="71" t="inlineStr">
         <is>
           <t>Machine learning 3: unsupervised learning and clustering</t>
         </is>
       </c>
-      <c r="C13" s="43">
+      <c r="C14" s="71">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/07-machine-learning-and-ai/README.md","Machine learning and AI literacy")</f>
         <v/>
       </c>
-      <c r="D13" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E13" s="43" t="inlineStr">
+      <c r="D14" s="72" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E14" s="71" t="inlineStr">
         <is>
           <t>Assignment 2</t>
         </is>
       </c>
-      <c r="F13" s="43" t="inlineStr">
+      <c r="F14" s="71" t="inlineStr">
         <is>
           <t>Assignment 1, before 4:00 PM</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="34" customHeight="1" s="35">
-      <c r="A14" s="54" t="n">
+    <row r="15" ht="34" customHeight="1" s="35">
+      <c r="A15" s="54" t="n">
         <v>46316</v>
       </c>
-      <c r="B14" s="40" t="inlineStr">
+      <c r="B15" s="40" t="inlineStr">
         <is>
           <t>Machine learning 4: forecasting, time series and anomalies</t>
         </is>
       </c>
-      <c r="C14" s="40">
+      <c r="C15" s="40">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/07-machine-learning-and-ai/README.md","Machine learning and AI literacy")</f>
         <v/>
       </c>
-      <c r="D14" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E14" s="40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" s="40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1" s="35">
-      <c r="A15" s="55" t="n">
+      <c r="D15" s="69" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E15" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F15" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1" s="35">
+      <c r="A16" s="81" t="n">
         <v>46320</v>
       </c>
-      <c r="B15" s="43" t="inlineStr">
+      <c r="B16" s="71" t="inlineStr">
         <is>
           <t>Machine learning 5: MLOps and what BigQuery ML gives you</t>
         </is>
       </c>
-      <c r="C15" s="43">
+      <c r="C16" s="71">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/07-machine-learning-and-ai/README.md","Machine learning and AI literacy")</f>
         <v/>
       </c>
-      <c r="D15" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E15" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F15" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1" s="35">
-      <c r="A16" s="56" t="n">
+      <c r="D16" s="72" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E16" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F16" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1" s="35">
+      <c r="A17" s="56" t="n">
         <v>46321</v>
       </c>
-      <c r="B16" s="40" t="inlineStr">
+      <c r="B17" s="40" t="inlineStr">
         <is>
           <t>Power BI Desktop and CSV data</t>
         </is>
       </c>
-      <c r="C16" s="40">
+      <c r="C17" s="40">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/03-power-query/README.md","Prepare data with Power Query")</f>
         <v/>
       </c>
-      <c r="D16" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E16" s="40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F16" s="40" t="inlineStr">
+      <c r="D17" s="69" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E17" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F17" s="40" t="inlineStr">
         <is>
           <t>Assignment 2, before 4:00 PM</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="34" customHeight="1" s="35">
-      <c r="A17" s="57" t="n">
+    <row r="18" ht="34" customHeight="1" s="35">
+      <c r="A18" s="82" t="n">
         <v>46324</v>
       </c>
-      <c r="B17" s="43" t="inlineStr">
+      <c r="B18" s="71" t="inlineStr">
         <is>
           <t>Power Query I: profile, clean and reshape files</t>
         </is>
       </c>
-      <c r="C17" s="43">
+      <c r="C18" s="71">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/03-power-query/README.md","Prepare data with Power Query")</f>
         <v/>
       </c>
-      <c r="D17" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E17" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="34" customHeight="1" s="35">
-      <c r="A18" s="58" t="n">
+      <c r="D18" s="72" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E18" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F18" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1" s="35">
+      <c r="A19" s="58" t="n">
         <v>46327</v>
       </c>
-      <c r="B18" s="40" t="inlineStr">
+      <c r="B19" s="40" t="inlineStr">
         <is>
           <t>Power Query II: combine queries and connect to BigQuery</t>
         </is>
       </c>
-      <c r="C18" s="40">
+      <c r="C19" s="40">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/03-power-query/README.md","Prepare data with Power Query")</f>
         <v/>
       </c>
-      <c r="D18" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E18" s="40" t="inlineStr">
+      <c r="D19" s="69" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E19" s="40" t="inlineStr">
         <is>
           <t>Assignment 3</t>
         </is>
       </c>
-      <c r="F18" s="40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="34" customHeight="1" s="35">
-      <c r="A19" s="59" t="n">
+      <c r="F19" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1" s="35">
+      <c r="A20" s="83" t="n">
         <v>46328</v>
       </c>
-      <c r="B19" s="43" t="inlineStr">
+      <c r="B20" s="71" t="inlineStr">
         <is>
           <t>Model: star schema, relationships and the date table</t>
         </is>
       </c>
-      <c r="C19" s="43">
+      <c r="C20" s="71">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/04-data-modeling-and-dax/README.md","Data modelling and DAX")</f>
         <v/>
       </c>
-      <c r="D19" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E19" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="34" customHeight="1" s="35">
-      <c r="A20" s="60" t="n">
+      <c r="D20" s="72" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E20" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1" s="35">
+      <c r="A21" s="60" t="n">
         <v>46329</v>
       </c>
-      <c r="B20" s="40" t="inlineStr">
+      <c r="B21" s="40" t="inlineStr">
         <is>
           <t>DAX I: measures and filter context</t>
         </is>
       </c>
-      <c r="C20" s="40">
+      <c r="C21" s="40">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/04-data-modeling-and-dax/README.md","Data modelling and DAX")</f>
         <v/>
       </c>
-      <c r="D20" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E20" s="40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="34" customHeight="1" s="35">
-      <c r="A21" s="61" t="n">
+      <c r="D21" s="69" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E21" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F21" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1" s="35">
+      <c r="A22" s="84" t="n">
         <v>46330</v>
       </c>
-      <c r="B21" s="43" t="inlineStr">
+      <c r="B22" s="71" t="inlineStr">
         <is>
           <t>DAX II: time and ranking</t>
         </is>
       </c>
-      <c r="C21" s="43">
+      <c r="C22" s="71">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/04-data-modeling-and-dax/README.md","Data modelling and DAX")</f>
         <v/>
       </c>
-      <c r="D21" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E21" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F21" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="34" customHeight="1" s="35">
-      <c r="A22" s="62" t="n">
+      <c r="D22" s="72" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E22" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F22" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1" s="35">
+      <c r="A23" s="62" t="n">
         <v>46331</v>
       </c>
-      <c r="B22" s="40" t="inlineStr">
+      <c r="B23" s="40" t="inlineStr">
         <is>
           <t>Report design and interactivity</t>
         </is>
       </c>
-      <c r="C22" s="40">
+      <c r="C23" s="40">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/05-visualization-and-storytelling/README.md","Visualisation and storytelling")</f>
         <v/>
       </c>
-      <c r="D22" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E22" s="40" t="inlineStr">
+      <c r="D23" s="69" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E23" s="40" t="inlineStr">
         <is>
           <t>Assignment 4</t>
         </is>
       </c>
-      <c r="F22" s="40" t="inlineStr">
+      <c r="F23" s="40" t="inlineStr">
         <is>
           <t>Assignment 3, before 4:00 PM</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="34" customHeight="1" s="35">
-      <c r="A23" s="63" t="n">
+    <row r="24" ht="34" customHeight="1" s="35">
+      <c r="A24" s="85" t="n">
         <v>46334</v>
       </c>
-      <c r="B23" s="43" t="inlineStr">
+      <c r="B24" s="71" t="inlineStr">
         <is>
           <t>Analyse and tell the story</t>
         </is>
       </c>
-      <c r="C23" s="43">
+      <c r="C24" s="71">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/05-visualization-and-storytelling/README.md","Visualisation and storytelling")</f>
         <v/>
       </c>
-      <c r="D23" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E23" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F23" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="34" customHeight="1" s="35">
-      <c r="A24" s="64" t="n">
+      <c r="D24" s="72" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E24" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1" s="35">
+      <c r="A25" s="64" t="n">
         <v>46335</v>
       </c>
-      <c r="B24" s="40" t="inlineStr">
+      <c r="B25" s="40" t="inlineStr">
         <is>
           <t>Manage and secure Power BI</t>
         </is>
       </c>
-      <c r="C24" s="40">
+      <c r="C25" s="40">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/06-power-bi-service/README.md","Manage and secure Power BI")</f>
         <v/>
       </c>
-      <c r="D24" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E24" s="40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F24" s="40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="34" customHeight="1" s="35">
-      <c r="A25" s="65" t="n">
+      <c r="D25" s="69" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E25" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F25" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1" s="35">
+      <c r="A26" s="86" t="n">
         <v>46336</v>
       </c>
-      <c r="B25" s="43" t="inlineStr">
+      <c r="B26" s="71" t="inlineStr">
         <is>
           <t>Generative AI for analysts</t>
         </is>
       </c>
-      <c r="C25" s="43">
+      <c r="C26" s="71">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/07-machine-learning-and-ai/README.md","Machine learning and AI literacy")</f>
         <v/>
       </c>
-      <c r="D25" s="41" t="inlineStr">
-        <is>
-          <t>After class</t>
-        </is>
-      </c>
-      <c r="E25" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" s="43" t="inlineStr">
+      <c r="D26" s="72" t="inlineStr">
+        <is>
+          <t>After class</t>
+        </is>
+      </c>
+      <c r="E26" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F26" s="71" t="inlineStr">
         <is>
           <t>Assignment 4, by 8:00 PM</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="34" customHeight="1" s="35">
-      <c r="A26" s="66" t="n">
+    <row r="27" ht="34" customHeight="1" s="35">
+      <c r="A27" s="66" t="n">
         <v>46337</v>
       </c>
-      <c r="B26" s="40" t="inlineStr">
+      <c r="B27" s="40" t="inlineStr">
         <is>
           <t>PL-300 review and weak-area clinic</t>
         </is>
       </c>
-      <c r="C26" s="40">
+      <c r="C27" s="40">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/08-pl300-and-career-readiness/README.md","PL-300 and career readiness")</f>
         <v/>
       </c>
-      <c r="D26" s="41" t="inlineStr">
+      <c r="D27" s="69" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E26" s="40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F26" s="40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1" s="35">
-      <c r="A27" s="67" t="n">
+      <c r="E27" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F27" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1" s="35">
+      <c r="A28" s="87" t="n">
         <v>46338</v>
       </c>
-      <c r="B27" s="43" t="inlineStr">
+      <c r="B28" s="71" t="inlineStr">
         <is>
           <t>Third-party mock and placement handoff</t>
         </is>
       </c>
-      <c r="C27" s="43">
+      <c r="C28" s="71">
         <f>HYPERLINK("https://github.com/tatwan/ASAC_Data_Science/blob/main/modules/08-pl300-and-career-readiness/README.md","PL-300 and career readiness")</f>
         <v/>
       </c>
-      <c r="D27" s="68" t="inlineStr">
+      <c r="D28" s="72" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E27" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F27" s="43" t="inlineStr">
+      <c r="E28" s="71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F28" s="71" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>